<commit_message>
backup before outbound_mixin refactor
</commit_message>
<xml_diff>
--- a/outbound/1_AAA_Allocation_CATL_202607.xlsx
+++ b/outbound/1_AAA_Allocation_CATL_202607.xlsx
@@ -487,7 +487,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="6" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
   </cols>
@@ -559,7 +559,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -568,11 +568,11 @@
         </is>
       </c>
       <c r="D3" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>1126011132</t>
+          <t>1126010723</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="J3" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="4">
@@ -616,11 +616,11 @@
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>1126011132</t>
+          <t>1126011233</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -644,7 +644,7 @@
         </is>
       </c>
       <c r="J4" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="5">
@@ -655,20 +655,20 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>1126011132</t>
+          <t>1126011511</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -692,7 +692,7 @@
         </is>
       </c>
       <c r="J5" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="6">
@@ -703,20 +703,20 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>1126011132</t>
+          <t>1126011511</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -740,7 +740,7 @@
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="7">
@@ -751,7 +751,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -760,11 +760,11 @@
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>1126011132</t>
+          <t>1126010634</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="J7" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="8">
@@ -799,7 +799,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -808,11 +808,11 @@
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>1126011132</t>
+          <t>1126010718</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -836,7 +836,7 @@
         </is>
       </c>
       <c r="J8" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="9">
@@ -847,7 +847,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -856,11 +856,11 @@
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>1126011132</t>
+          <t>1126010718</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -884,7 +884,7 @@
         </is>
       </c>
       <c r="J9" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="10">
@@ -895,7 +895,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -904,11 +904,11 @@
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>1126011132</t>
+          <t>1125122364</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -932,7 +932,7 @@
         </is>
       </c>
       <c r="J10" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="11">
@@ -943,7 +943,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -952,11 +952,11 @@
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>1126011132</t>
+          <t>1126010934</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -980,7 +980,7 @@
         </is>
       </c>
       <c r="J11" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="12">
@@ -991,7 +991,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1000,11 +1000,11 @@
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>1126011132</t>
+          <t>1126010635</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -1028,7 +1028,7 @@
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="13">
@@ -1048,11 +1048,11 @@
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>1126011136</t>
+          <t>1126011232</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="14">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1096,11 +1096,11 @@
         </is>
       </c>
       <c r="D14" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>1126011136</t>
+          <t>1126010636</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="15">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1144,11 +1144,11 @@
         </is>
       </c>
       <c r="D15" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>1126011136</t>
+          <t>1125122363</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -1172,7 +1172,7 @@
         </is>
       </c>
       <c r="J15" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="16">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1192,11 +1192,11 @@
         </is>
       </c>
       <c r="D16" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>1126011136</t>
+          <t>1125122363</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="17">
@@ -1240,11 +1240,11 @@
         </is>
       </c>
       <c r="D17" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>1126011136</t>
+          <t>1126011131</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1268,7 +1268,7 @@
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="18">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -1288,11 +1288,11 @@
         </is>
       </c>
       <c r="D18" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>1126011136</t>
+          <t>1126010637</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1316,7 +1316,7 @@
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="19">
@@ -1327,20 +1327,20 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D19" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>1126011136</t>
+          <t>1126011446</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1364,7 +1364,7 @@
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="20">
@@ -1384,11 +1384,11 @@
         </is>
       </c>
       <c r="D20" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>1126011136</t>
+          <t>1126011538</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1412,7 +1412,7 @@
         </is>
       </c>
       <c r="J20" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="21">
@@ -1432,11 +1432,11 @@
         </is>
       </c>
       <c r="D21" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>1126011136</t>
+          <t>1126011213</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="22">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1480,11 +1480,11 @@
         </is>
       </c>
       <c r="D22" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>1126011136</t>
+          <t>1126010702</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -1508,7 +1508,7 @@
         </is>
       </c>
       <c r="J22" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="23">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>2200034274</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1528,11 +1528,11 @@
         </is>
       </c>
       <c r="D23" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>1126010737</t>
+          <t>1126010702</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -1556,7 +1556,7 @@
         </is>
       </c>
       <c r="J23" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="24">
@@ -1576,11 +1576,11 @@
         </is>
       </c>
       <c r="D24" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>1126010737</t>
+          <t>1126010933</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -1604,7 +1604,7 @@
         </is>
       </c>
       <c r="J24" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="25">
@@ -1624,11 +1624,11 @@
         </is>
       </c>
       <c r="D25" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>1126010737</t>
+          <t>1126010933</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -1652,7 +1652,7 @@
         </is>
       </c>
       <c r="J25" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="26">
@@ -1663,7 +1663,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>2200034274</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -1672,11 +1672,11 @@
         </is>
       </c>
       <c r="D26" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>1126010737</t>
+          <t>1126010643</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -1700,7 +1700,7 @@
         </is>
       </c>
       <c r="J26" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="27">
@@ -1720,11 +1720,11 @@
         </is>
       </c>
       <c r="D27" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>1126010737</t>
+          <t>1126010932</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -1748,7 +1748,7 @@
         </is>
       </c>
       <c r="J27" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="28">
@@ -1768,11 +1768,11 @@
         </is>
       </c>
       <c r="D28" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>1126010737</t>
+          <t>1126010932</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -1796,7 +1796,7 @@
         </is>
       </c>
       <c r="J28" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="29">
@@ -1807,7 +1807,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>2200034274</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -1816,11 +1816,11 @@
         </is>
       </c>
       <c r="D29" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>1126010737</t>
+          <t>1126011132</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -1844,7 +1844,7 @@
         </is>
       </c>
       <c r="J29" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="30">
@@ -1855,7 +1855,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>2200034274</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -1864,11 +1864,11 @@
         </is>
       </c>
       <c r="D30" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>1126010737</t>
+          <t>1126011132</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -1892,7 +1892,7 @@
         </is>
       </c>
       <c r="J30" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="31">
@@ -1912,11 +1912,11 @@
         </is>
       </c>
       <c r="D31" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>1126010737</t>
+          <t>1126010804</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -1940,7 +1940,7 @@
         </is>
       </c>
       <c r="J31" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="32">
@@ -1951,7 +1951,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>2200034274</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -1960,11 +1960,11 @@
         </is>
       </c>
       <c r="D32" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>1126010737</t>
+          <t>1126010720</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -1988,7 +1988,7 @@
         </is>
       </c>
       <c r="J32" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="33">
@@ -2008,11 +2008,11 @@
         </is>
       </c>
       <c r="D33" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>1126010721</t>
+          <t>1126010720</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -2036,7 +2036,7 @@
         </is>
       </c>
       <c r="J33" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="34">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -2056,11 +2056,11 @@
         </is>
       </c>
       <c r="D34" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>1126010721</t>
+          <t>1126010801</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -2084,7 +2084,7 @@
         </is>
       </c>
       <c r="J34" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="35">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -2104,11 +2104,11 @@
         </is>
       </c>
       <c r="D35" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>1126010721</t>
+          <t>1126011212</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
@@ -2132,7 +2132,7 @@
         </is>
       </c>
       <c r="J35" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="36">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -2152,11 +2152,11 @@
         </is>
       </c>
       <c r="D36" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>1126010721</t>
+          <t>1126011112</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
@@ -2180,7 +2180,7 @@
         </is>
       </c>
       <c r="J36" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="37">
@@ -2200,11 +2200,11 @@
         </is>
       </c>
       <c r="D37" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>1126010721</t>
+          <t>1126010703</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
@@ -2228,7 +2228,7 @@
         </is>
       </c>
       <c r="J37" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="38">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -2248,11 +2248,11 @@
         </is>
       </c>
       <c r="D38" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>1126010721</t>
+          <t>1126011128</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
@@ -2276,7 +2276,7 @@
         </is>
       </c>
       <c r="J38" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="39">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -2296,11 +2296,11 @@
         </is>
       </c>
       <c r="D39" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>1126010721</t>
+          <t>1126011128</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
@@ -2324,7 +2324,7 @@
         </is>
       </c>
       <c r="J39" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="40">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -2344,11 +2344,11 @@
         </is>
       </c>
       <c r="D40" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>1126010721</t>
+          <t>1126010379</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -2372,7 +2372,7 @@
         </is>
       </c>
       <c r="J40" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="41">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -2392,11 +2392,11 @@
         </is>
       </c>
       <c r="D41" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>1126010721</t>
+          <t>1126010379</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
@@ -2420,7 +2420,7 @@
         </is>
       </c>
       <c r="J41" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="42">
@@ -2431,7 +2431,7 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -2440,11 +2440,11 @@
         </is>
       </c>
       <c r="D42" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>1126010721</t>
+          <t>1126011117</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
@@ -2468,7 +2468,7 @@
         </is>
       </c>
       <c r="J42" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="43">
@@ -2479,7 +2479,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -2488,11 +2488,11 @@
         </is>
       </c>
       <c r="D43" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>1126010645</t>
+          <t>1126011117</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
@@ -2516,7 +2516,7 @@
         </is>
       </c>
       <c r="J43" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="44">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -2536,11 +2536,11 @@
         </is>
       </c>
       <c r="D44" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>1126010645</t>
+          <t>1126011130</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -2564,7 +2564,7 @@
         </is>
       </c>
       <c r="J44" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="45">
@@ -2575,7 +2575,7 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -2584,11 +2584,11 @@
         </is>
       </c>
       <c r="D45" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>1126010645</t>
+          <t>1126010821</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
@@ -2612,7 +2612,7 @@
         </is>
       </c>
       <c r="J45" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="46">
@@ -2623,7 +2623,7 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -2632,11 +2632,11 @@
         </is>
       </c>
       <c r="D46" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>1126010645</t>
+          <t>1126010821</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
@@ -2660,7 +2660,7 @@
         </is>
       </c>
       <c r="J46" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="47">
@@ -2671,7 +2671,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -2680,11 +2680,11 @@
         </is>
       </c>
       <c r="D47" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>1126010645</t>
+          <t>1126010803</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
@@ -2708,7 +2708,7 @@
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="48">
@@ -2719,7 +2719,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -2728,11 +2728,11 @@
         </is>
       </c>
       <c r="D48" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>1126010645</t>
+          <t>1126010803</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
@@ -2756,7 +2756,7 @@
         </is>
       </c>
       <c r="J48" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="49">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -2776,11 +2776,11 @@
         </is>
       </c>
       <c r="D49" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>1126010645</t>
+          <t>1126010719</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
@@ -2804,7 +2804,7 @@
         </is>
       </c>
       <c r="J49" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="50">
@@ -2815,7 +2815,7 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -2824,11 +2824,11 @@
         </is>
       </c>
       <c r="D50" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>1126010645</t>
+          <t>1126010719</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
@@ -2852,7 +2852,7 @@
         </is>
       </c>
       <c r="J50" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="51">
@@ -2863,20 +2863,20 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D51" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>1126010645</t>
+          <t>1126011510</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
@@ -2900,7 +2900,7 @@
         </is>
       </c>
       <c r="J51" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="52">
@@ -2911,20 +2911,20 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D52" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>1126010645</t>
+          <t>1126011510</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
@@ -2948,7 +2948,7 @@
         </is>
       </c>
       <c r="J52" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="53">
@@ -2959,7 +2959,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -2968,11 +2968,11 @@
         </is>
       </c>
       <c r="D53" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>1126010717</t>
+          <t>1126010814</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
@@ -2996,7 +2996,7 @@
         </is>
       </c>
       <c r="J53" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="54">
@@ -3007,7 +3007,7 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
@@ -3016,11 +3016,11 @@
         </is>
       </c>
       <c r="D54" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>1126010717</t>
+          <t>1126010814</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
@@ -3044,7 +3044,7 @@
         </is>
       </c>
       <c r="J54" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="55">
@@ -3055,7 +3055,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -3064,11 +3064,11 @@
         </is>
       </c>
       <c r="D55" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>1126010717</t>
+          <t>1126011118</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
@@ -3092,7 +3092,7 @@
         </is>
       </c>
       <c r="J55" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="56">
@@ -3103,7 +3103,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -3112,11 +3112,11 @@
         </is>
       </c>
       <c r="D56" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>1126010717</t>
+          <t>1126011118</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
@@ -3140,7 +3140,7 @@
         </is>
       </c>
       <c r="J56" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="57">
@@ -3151,7 +3151,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -3160,11 +3160,11 @@
         </is>
       </c>
       <c r="D57" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>1126010717</t>
+          <t>1126011134</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
@@ -3188,7 +3188,7 @@
         </is>
       </c>
       <c r="J57" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="58">
@@ -3199,7 +3199,7 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
@@ -3208,11 +3208,11 @@
         </is>
       </c>
       <c r="D58" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>1126010717</t>
+          <t>1126010240</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J58" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="59">
@@ -3256,11 +3256,11 @@
         </is>
       </c>
       <c r="D59" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>1126010717</t>
+          <t>1126010638</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
@@ -3284,7 +3284,7 @@
         </is>
       </c>
       <c r="J59" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="60">
@@ -3295,20 +3295,20 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D60" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>1126010717</t>
+          <t>1126011531</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
@@ -3332,7 +3332,7 @@
         </is>
       </c>
       <c r="J60" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="61">
@@ -3352,11 +3352,11 @@
         </is>
       </c>
       <c r="D61" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>1126010717</t>
+          <t>1126010639</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
@@ -3380,7 +3380,7 @@
         </is>
       </c>
       <c r="J61" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="62">
@@ -3391,20 +3391,20 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D62" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>1126010717</t>
+          <t>1126011504</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
@@ -3428,7 +3428,7 @@
         </is>
       </c>
       <c r="J62" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="63">
@@ -3448,11 +3448,11 @@
         </is>
       </c>
       <c r="D63" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>1126010932</t>
+          <t>1126010739</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
@@ -3476,7 +3476,7 @@
         </is>
       </c>
       <c r="J63" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="64">
@@ -3496,11 +3496,11 @@
         </is>
       </c>
       <c r="D64" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>1126010932</t>
+          <t>1126010739</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="J64" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="65">
@@ -3535,7 +3535,7 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>2200034274</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -3544,11 +3544,11 @@
         </is>
       </c>
       <c r="D65" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>1126010932</t>
+          <t>1126010642</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
@@ -3572,7 +3572,7 @@
         </is>
       </c>
       <c r="J65" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="66">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>2200034274</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
@@ -3592,11 +3592,11 @@
         </is>
       </c>
       <c r="D66" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>1126010932</t>
+          <t>1126011211</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
@@ -3620,7 +3620,7 @@
         </is>
       </c>
       <c r="J66" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="67">
@@ -3631,7 +3631,7 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>2200034274</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
@@ -3640,11 +3640,11 @@
         </is>
       </c>
       <c r="D67" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>1126010932</t>
+          <t>1126011211</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
@@ -3668,7 +3668,7 @@
         </is>
       </c>
       <c r="J67" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="68">
@@ -3679,20 +3679,20 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>2200034274</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D68" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>1126010932</t>
+          <t>1126011442</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
@@ -3716,7 +3716,7 @@
         </is>
       </c>
       <c r="J68" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="69">
@@ -3727,7 +3727,7 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>2200034274</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
@@ -3736,11 +3736,11 @@
         </is>
       </c>
       <c r="D69" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>1126010932</t>
+          <t>1126010378</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
@@ -3764,7 +3764,7 @@
         </is>
       </c>
       <c r="J69" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="70">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>2200034274</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
@@ -3784,11 +3784,11 @@
         </is>
       </c>
       <c r="D70" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>1126010932</t>
+          <t>1126010378</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
@@ -3812,7 +3812,7 @@
         </is>
       </c>
       <c r="J70" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="71">
@@ -3823,20 +3823,20 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>2200034274</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D71" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>1126010932</t>
+          <t>1126010548</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
@@ -3860,7 +3860,7 @@
         </is>
       </c>
       <c r="J71" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="72">
@@ -3871,7 +3871,7 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>2200034274</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
@@ -3880,11 +3880,11 @@
         </is>
       </c>
       <c r="D72" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>1126010932</t>
+          <t>1126011537</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
@@ -3908,7 +3908,7 @@
         </is>
       </c>
       <c r="J72" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="73">
@@ -3919,7 +3919,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
@@ -3928,11 +3928,11 @@
         </is>
       </c>
       <c r="D73" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>1126011213</t>
+          <t>1126010812</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
@@ -3956,7 +3956,7 @@
         </is>
       </c>
       <c r="J73" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="74">
@@ -3967,7 +3967,7 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
@@ -3976,11 +3976,11 @@
         </is>
       </c>
       <c r="D74" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>1126011213</t>
+          <t>1126010812</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
@@ -4004,7 +4004,7 @@
         </is>
       </c>
       <c r="J74" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="75">
@@ -4015,7 +4015,7 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -4024,11 +4024,11 @@
         </is>
       </c>
       <c r="D75" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>1126011213</t>
+          <t>1126010706</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
@@ -4052,7 +4052,7 @@
         </is>
       </c>
       <c r="J75" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="76">
@@ -4063,7 +4063,7 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -4072,11 +4072,11 @@
         </is>
       </c>
       <c r="D76" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>1126011213</t>
+          <t>1126010706</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
@@ -4100,7 +4100,7 @@
         </is>
       </c>
       <c r="J76" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="77">
@@ -4111,7 +4111,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -4120,11 +4120,11 @@
         </is>
       </c>
       <c r="D77" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>1126011213</t>
+          <t>1126011015</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
@@ -4148,7 +4148,7 @@
         </is>
       </c>
       <c r="J77" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="78">
@@ -4159,20 +4159,20 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D78" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>1126011213</t>
+          <t>1126011445</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
@@ -4196,7 +4196,7 @@
         </is>
       </c>
       <c r="J78" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="79">
@@ -4207,20 +4207,20 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D79" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>1126011213</t>
+          <t>1126011534</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
@@ -4244,7 +4244,7 @@
         </is>
       </c>
       <c r="J79" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="80">
@@ -4255,20 +4255,20 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D80" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>1126011213</t>
+          <t>1126011534</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
@@ -4292,7 +4292,7 @@
         </is>
       </c>
       <c r="J80" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="81">
@@ -4303,7 +4303,7 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
@@ -4312,11 +4312,11 @@
         </is>
       </c>
       <c r="D81" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>1126011213</t>
+          <t>1126010705</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
@@ -4340,7 +4340,7 @@
         </is>
       </c>
       <c r="J81" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="82">
@@ -4360,11 +4360,11 @@
         </is>
       </c>
       <c r="D82" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>1126011213</t>
+          <t>1126011136</t>
         </is>
       </c>
       <c r="F82" s="3" t="inlineStr">
@@ -4388,7 +4388,7 @@
         </is>
       </c>
       <c r="J82" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="83">
@@ -4399,7 +4399,7 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -4408,11 +4408,11 @@
         </is>
       </c>
       <c r="D83" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>1126010641</t>
+          <t>1126010151</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
@@ -4436,7 +4436,7 @@
         </is>
       </c>
       <c r="J83" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="84">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
@@ -4456,11 +4456,11 @@
         </is>
       </c>
       <c r="D84" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>1126010641</t>
+          <t>1126010740</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
@@ -4484,7 +4484,7 @@
         </is>
       </c>
       <c r="J84" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="85">
@@ -4495,7 +4495,7 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -4504,11 +4504,11 @@
         </is>
       </c>
       <c r="D85" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>1126010641</t>
+          <t>1126010740</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
@@ -4532,7 +4532,7 @@
         </is>
       </c>
       <c r="J85" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="86">
@@ -4543,20 +4543,20 @@
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D86" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>1126010641</t>
+          <t>1125110452</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
@@ -4580,7 +4580,7 @@
         </is>
       </c>
       <c r="J86" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="87">
@@ -4591,7 +4591,7 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -4600,11 +4600,11 @@
         </is>
       </c>
       <c r="D87" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>1126010641</t>
+          <t>1126011209</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
@@ -4628,7 +4628,7 @@
         </is>
       </c>
       <c r="J87" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="88">
@@ -4639,20 +4639,20 @@
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D88" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>1126010641</t>
+          <t>1126011509</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
@@ -4676,7 +4676,7 @@
         </is>
       </c>
       <c r="J88" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="89">
@@ -4687,20 +4687,20 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D89" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>1126010641</t>
+          <t>1126011509</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
@@ -4724,7 +4724,7 @@
         </is>
       </c>
       <c r="J89" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="90">
@@ -4744,11 +4744,11 @@
         </is>
       </c>
       <c r="D90" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>1126010641</t>
+          <t>1126010644</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
@@ -4772,7 +4772,7 @@
         </is>
       </c>
       <c r="J90" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="91">
@@ -4783,20 +4783,20 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D91" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>1126010641</t>
+          <t>1126011535</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
@@ -4820,7 +4820,7 @@
         </is>
       </c>
       <c r="J91" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="92">
@@ -4831,20 +4831,20 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D92" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>1126010641</t>
+          <t>1126011535</t>
         </is>
       </c>
       <c r="F92" s="3" t="inlineStr">
@@ -4868,7 +4868,7 @@
         </is>
       </c>
       <c r="J92" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="93">
@@ -4879,20 +4879,20 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D93" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>1126011211</t>
+          <t>1126011505</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
@@ -4916,7 +4916,7 @@
         </is>
       </c>
       <c r="J93" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="94">
@@ -4927,20 +4927,20 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D94" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>1126011211</t>
+          <t>1126011505</t>
         </is>
       </c>
       <c r="F94" s="3" t="inlineStr">
@@ -4964,7 +4964,7 @@
         </is>
       </c>
       <c r="J94" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="95">
@@ -4975,20 +4975,20 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D95" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>1126011211</t>
+          <t>1126011432</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
@@ -5012,7 +5012,7 @@
         </is>
       </c>
       <c r="J95" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="96">
@@ -5023,20 +5023,20 @@
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D96" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>1126011211</t>
+          <t>1126011432</t>
         </is>
       </c>
       <c r="F96" s="3" t="inlineStr">
@@ -5060,7 +5060,7 @@
         </is>
       </c>
       <c r="J96" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="97">
@@ -5071,7 +5071,7 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
@@ -5080,11 +5080,11 @@
         </is>
       </c>
       <c r="D97" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>1126011211</t>
+          <t>1126011133</t>
         </is>
       </c>
       <c r="F97" s="3" t="inlineStr">
@@ -5108,7 +5108,7 @@
         </is>
       </c>
       <c r="J97" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="98">
@@ -5119,7 +5119,7 @@
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
@@ -5128,11 +5128,11 @@
         </is>
       </c>
       <c r="D98" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>1126011211</t>
+          <t>1126011133</t>
         </is>
       </c>
       <c r="F98" s="3" t="inlineStr">
@@ -5156,7 +5156,7 @@
         </is>
       </c>
       <c r="J98" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="99">
@@ -5167,7 +5167,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -5176,11 +5176,11 @@
         </is>
       </c>
       <c r="D99" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>1126011211</t>
+          <t>1126010802</t>
         </is>
       </c>
       <c r="F99" s="3" t="inlineStr">
@@ -5204,7 +5204,7 @@
         </is>
       </c>
       <c r="J99" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="100">
@@ -5215,7 +5215,7 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
@@ -5224,11 +5224,11 @@
         </is>
       </c>
       <c r="D100" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>1126011211</t>
+          <t>1126010802</t>
         </is>
       </c>
       <c r="F100" s="3" t="inlineStr">
@@ -5252,7 +5252,7 @@
         </is>
       </c>
       <c r="J100" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="101">
@@ -5263,7 +5263,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -5272,11 +5272,11 @@
         </is>
       </c>
       <c r="D101" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>1126011211</t>
+          <t>1126010640</t>
         </is>
       </c>
       <c r="F101" s="3" t="inlineStr">
@@ -5300,7 +5300,7 @@
         </is>
       </c>
       <c r="J101" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="102">
@@ -5311,7 +5311,7 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
@@ -5320,11 +5320,11 @@
         </is>
       </c>
       <c r="D102" s="4" t="n">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>1126011211</t>
+          <t>1126010640</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
@@ -5348,7 +5348,7 @@
         </is>
       </c>
       <c r="J102" s="4" t="n">
-        <v>5.13</v>
+        <v>0.513</v>
       </c>
     </row>
     <row r="103">
@@ -5359,7 +5359,7 @@
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034274</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
@@ -5372,7 +5372,7 @@
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t>1126011132</t>
+          <t>1126010723</t>
         </is>
       </c>
       <c r="F103" s="5" t="inlineStr">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="E104" s="5" t="inlineStr">
         <is>
-          <t>1126011136</t>
+          <t>1126011233</t>
         </is>
       </c>
       <c r="F104" s="5" t="inlineStr">
@@ -5455,12 +5455,12 @@
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>2200034274</t>
+          <t>2200034275</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>2026-03-21</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="D105" s="6" t="n">
@@ -5468,7 +5468,7 @@
       </c>
       <c r="E105" s="5" t="inlineStr">
         <is>
-          <t>1126010737</t>
+          <t>1126011511</t>
         </is>
       </c>
       <c r="F105" s="5" t="inlineStr">
@@ -5516,7 +5516,7 @@
       </c>
       <c r="E106" s="5" t="inlineStr">
         <is>
-          <t>1126010721</t>
+          <t>1126010634</t>
         </is>
       </c>
       <c r="F106" s="5" t="inlineStr">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="E107" s="5" t="inlineStr">
         <is>
-          <t>1126010645</t>
+          <t>1126010718</t>
         </is>
       </c>
       <c r="F107" s="5" t="inlineStr">
@@ -5612,7 +5612,7 @@
       </c>
       <c r="E108" s="5" t="inlineStr">
         <is>
-          <t>1126010717</t>
+          <t>1125122364</t>
         </is>
       </c>
       <c r="F108" s="5" t="inlineStr">
@@ -5660,7 +5660,7 @@
       </c>
       <c r="E109" s="5" t="inlineStr">
         <is>
-          <t>1126010932</t>
+          <t>1126010934</t>
         </is>
       </c>
       <c r="F109" s="5" t="inlineStr">
@@ -5695,7 +5695,7 @@
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="E110" s="5" t="inlineStr">
         <is>
-          <t>1126011213</t>
+          <t>1126010635</t>
         </is>
       </c>
       <c r="F110" s="5" t="inlineStr">
@@ -5743,7 +5743,7 @@
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>2200034273</t>
+          <t>2200034276</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
@@ -5756,7 +5756,7 @@
       </c>
       <c r="E111" s="5" t="inlineStr">
         <is>
-          <t>1126010641</t>
+          <t>1126011232</t>
         </is>
       </c>
       <c r="F111" s="5" t="inlineStr">
@@ -5791,7 +5791,7 @@
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>2200034276</t>
+          <t>2200034273</t>
         </is>
       </c>
       <c r="C112" s="5" t="inlineStr">
@@ -5804,7 +5804,7 @@
       </c>
       <c r="E112" s="5" t="inlineStr">
         <is>
-          <t>1126011211</t>
+          <t>1126010636</t>
         </is>
       </c>
       <c r="F112" s="5" t="inlineStr">

</xml_diff>